<commit_message>
Update soccer trades 2026-08-07 17:02:25 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Division Profesional/trades.xlsx
+++ b/data/sxbet/ligas/Division Profesional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.42</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786117945</t>
+          <t>1786120674</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>24.427807</t>
+          <t>4.727273</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12.82</t>
+          <t>1.65998</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786116567</t>
+          <t>1786119912</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>27.718919</t>
+          <t>2.25082</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.27945</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,24 +785,24 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano 0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -810,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>8.616741</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.31576</t>
+          <t>17.6089</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.3662</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1.5</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -914,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>8.616781</t>
+          <t>48.078908</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +979,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,12 +994,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>27.21968</t>
+          <t>33.06999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.7338</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1056,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786116497</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>37.35119</t>
+          <t>45.069833</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1091,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.0374</t>
+          <t>22.48</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.4675</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1130,7 +1146,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786116493</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>37.348465</t>
+          <t>48.085561</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,12 +1203,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1202,22 +1218,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>28.42</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Academia De Balompie Boliviano -0.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1227,27 +1243,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,17 +1288,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786116236</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>62.947368</t>
+          <t>48.067653</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,31 +1315,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>11.42</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5075</t>
+          <t>1.4675</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1331,27 +1355,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1400,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786116231</t>
+          <t>1786117945</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>79.82266</t>
+          <t>24.427807</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,7 +1427,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1418,39 +1442,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.85998</t>
+          <t>12.82</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.4625</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -1458,7 +1482,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1488,7 +1512,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786115704</t>
+          <t>1786116567</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1522,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2.56549</t>
+          <t>27.718919</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,110 +1539,870 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>6.27945</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>8.616741</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2.31576</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>8.616781</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>27.21968</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786116497</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>37.35119</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>10.0374</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786116493</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>37.348465</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>17.94</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786116236</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>62.947368</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.5075</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786116231</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>79.82266</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.85998</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.725</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786115704</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2.56549</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>0x590b15150f41ddf420690c7cecb635a5facfe4448334123e390e09254607c190</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>9.19</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>1.3562</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Guabira</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>L19682540</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>1786115704</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>1786137300</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>25.796491</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 19:02:53 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Division Profesional/trades.xlsx
+++ b/data/sxbet/ligas/Division Profesional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
+          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,46 +539,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7425</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786120674</t>
+          <t>1786127516</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4.727273</t>
+          <t>7.111111</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
+          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,46 +643,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.65998</t>
+          <t>5.75999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7375</t>
+          <t>1.8113</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -698,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786119912</t>
+          <t>1786127077</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2.25082</t>
+          <t>7.100142</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,12 +754,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>9.99</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,7 +769,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano 0</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126518</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>13.32</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,22 +866,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17.6089</t>
+          <t>8.36115</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3662</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1.5</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -922,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>48.078908</t>
+          <t>11.204221</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,27 +963,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>33.06999</t>
+          <t>2.81507</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.7338</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1007,26 +987,22 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -1064,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>45.069833</t>
+          <t>11.204259</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,12 +1067,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1106,22 +1082,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22.48</t>
+          <t>27.87055</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1146,7 +1122,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1176,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1186,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>48.085561</t>
+          <t>37.347471</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,39 +1179,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>9.38356</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano -0.5</t>
-        </is>
-      </c>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1258,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1288,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.067653</t>
+          <t>37.347502</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,12 +1283,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1330,22 +1298,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11.42</t>
+          <t>12.87</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1370,7 +1338,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1400,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786117945</t>
+          <t>1786125953</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1410,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>24.427807</t>
+          <t>17.16</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1427,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1442,12 +1410,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>12.82</t>
+          <t>5.82</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1457,7 +1425,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1467,27 +1435,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1512,17 +1480,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786116567</t>
+          <t>1786124724</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>27.718919</t>
+          <t>15.836735</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1539,12 +1507,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1554,12 +1522,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6.27945</t>
+          <t>1.93998</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1624,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786124628</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1634,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>8.616741</t>
+          <t>2.58664</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1651,23 +1619,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.31576</t>
+          <t>3.55998</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1675,7 +1647,11 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1728,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786124356</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1738,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>8.616781</t>
+          <t>4.74664</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1755,12 +1731,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1770,22 +1746,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>27.21968</t>
+          <t>8.94</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1795,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1840,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786116497</t>
+          <t>1786123837</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>37.35119</t>
+          <t>24.080808</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1867,31 +1843,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.0374</t>
+          <t>17.66906</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Real Tomayapo -1</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1899,27 +1883,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1944,17 +1928,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786116493</t>
+          <t>1786123806</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>37.348465</t>
+          <t>48.079075</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1971,7 +1955,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1979,54 +1963,46 @@
           <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>27.12529</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>Real Oruro</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Real Tomayapo vs Real Oruro</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Real Tomayapo</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Real Oruro</t>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2056,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786116236</t>
+          <t>1786123085</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2066,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>62.947368</t>
+          <t>54.115292</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2083,31 +2059,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5075</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2115,27 +2099,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2160,17 +2144,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786116231</t>
+          <t>1786120674</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>79.82266</t>
+          <t>4.727273</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2187,7 +2171,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2202,12 +2186,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.85998</t>
+          <t>1.65998</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2272,7 +2256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786115704</t>
+          <t>1786119912</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2282,7 +2266,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2.56549</t>
+          <t>2.25082</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2299,110 +2283,1654 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano 0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>17.6089</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.3662</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>48.078908</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>33.06999</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.7338</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>45.069833</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>22.48</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.4675</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1786118874</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>48.085561</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>28.42</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.5913</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -0.5</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1786118874</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>48.067653</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>11.42</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.4675</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1786117945</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>24.427807</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>12.82</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786116567</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>27.718919</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>6.27945</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>8.616741</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2.31576</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>8.616781</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>27.21968</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786116497</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>37.35119</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>10.0374</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786116493</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>37.348465</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>17.94</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786116236</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>62.947368</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.5075</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1786116231</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>79.82266</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1.85998</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.725</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1786115704</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>2.56549</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>0x590b15150f41ddf420690c7cecb635a5facfe4448334123e390e09254607c190</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>9.19</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>1.3562</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Guabira</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>L19682540</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
         <is>
           <t>1786115704</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S32" t="inlineStr">
         <is>
           <t>1786137300</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>25.796491</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-07 21:03:18 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Division Profesional/trades.xlsx
+++ b/data/sxbet/ligas/Division Profesional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V32"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
+          <t>0x665ad5dc09f910a78682d8cac57b8941da70edf35f23f2fb6db3f128b63a18e8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>11.31</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786127516</t>
+          <t>1786136236</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>7.111111</t>
+          <t>19.374732</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,31 +635,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
+          <t>0xf272c06e82de6d4f5a541673d36a6677e813d924b288c8fa65932e7f17a6e89f</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.75999</t>
+          <t>33.32</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.8113</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -682,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786127077</t>
+          <t>1786136032</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>7.100142</t>
+          <t>60.307692</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
+          <t>0x0a6830dca2ddaafc8a77ba73c5db8e87d8f5fbc96d7d4d1fc85c80dd6a2dcff0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -747,31 +755,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9.99</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -779,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786126518</t>
+          <t>1786135821</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>13.32</t>
+          <t>13.395349</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,54 +851,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
+          <t>0x1b16769a2446e95c5c45c0a5c1eee6a448ebe2fc2e9b698f501443da0dfe730a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.36115</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.7462</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -906,7 +898,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786135233</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>11.204221</t>
+          <t>8.961131</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,28 +955,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
+          <t>0x3b7d6449f4a2a7f7e958feb31d1aa3512a36d932b93cd01aba4dae26404c5131</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.81507</t>
+          <t>17.00737</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2512</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1010,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1040,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786134933</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>11.204259</t>
+          <t>48.077371</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,39 +1059,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
+          <t>0x5b2bf2a561f9efc207b4be16204e262143fe9b1140ba536a8207f25e53ad496b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>27.87055</t>
+          <t>2.22</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7462</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1107,27 +1091,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1152,17 +1136,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786134605</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>37.347471</t>
+          <t>5.431193</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,31 +1163,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
+          <t>0xcc60eac075cc4315d4dfa294b65cc4f174c2c9d458811a16d52e87b659d8ad45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.38356</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2512</t>
+          <t>1.5362</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1226,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786134304</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>37.347502</t>
+          <t>9.323991</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,12 +1275,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
+          <t>0xe21791ae1e8109a191bcf87ea7e050cf62a2cdf8ddab67d9bf182b3016b1b848</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1298,39 +1290,39 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12.87</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -1338,7 +1330,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1368,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786125953</t>
+          <t>1786134118</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>17.16</t>
+          <t>49.767221</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1387,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
+          <t>0xc3316b5940ad1bd194feda7f00770a34f912831f1c7deace747e91137cafd11b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1410,22 +1402,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5.82</t>
+          <t>15.16819</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3125</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1435,27 +1427,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0x48f1daf9c9d3e68c0ec6553b26f71366417addfa8f09d543cc8f8bdd0077b612</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,17 +1472,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786124724</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>15.836735</t>
+          <t>48.538208</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1499,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
+          <t>0x3c412198bcfc31cf640052941892a1f595f5547ec59a1414e24fbb1bfeb3ebae</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1522,39 +1514,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.93998</t>
+          <t>18.5095</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -1562,7 +1554,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x2f4dc11491614174f697fd6856dc7dfbde0374f56c9c6b93da705d898b6b9392</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1592,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786124628</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2.58664</t>
+          <t>48.549508</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
+          <t>0x2cb6bec7f2a474ec0b4c474043876d18add5eadb31632382e7e9f728fa247159</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1634,39 +1626,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.55998</t>
+          <t>15.66</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.6425</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -1674,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1704,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786124356</t>
+          <t>1786131081</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1714,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>4.74664</t>
+          <t>24.373541</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1723,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
+          <t>0x2a44ccf443a8d5632916aab67a3e7bc4147a268fe5d4978cedf712cfd7e2babf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,22 +1738,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.94</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1771,27 +1763,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>San Antonio Bulo Bulo</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19691489</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1808,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786123837</t>
+          <t>1786130177</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>24.080808</t>
+          <t>2.605863</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,12 +1835,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
+          <t>0x116fd7242c980c72161b884392f42af79732e449e79f3dc7d212acd8ad8d658d</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1858,22 +1850,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17.66906</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1883,27 +1875,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1928,17 +1920,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786123806</t>
+          <t>1786129447</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>48.079075</t>
+          <t>9.82799</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1955,28 +1947,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
+          <t>0xbbe9c61e5707bbf256b5c277314eeffa098594034d2dbb2bb99c6791f780e113</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>27.12529</t>
+          <t>7.35999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1987,27 +1979,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>San Antonio Bulo Bulo</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
+          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19691489</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2032,17 +2024,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786123085</t>
+          <t>1786129377</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>54.115292</t>
+          <t>9.945932</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,7 +2051,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
+          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2067,46 +2059,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.7425</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2114,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2144,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786120674</t>
+          <t>1786127516</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>4.727273</t>
+          <t>7.111111</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,7 +2155,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
+          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2179,46 +2163,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.65998</t>
+          <t>5.75999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7375</t>
+          <t>1.8113</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2226,7 +2202,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2256,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786119912</t>
+          <t>1786127077</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2266,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2.25082</t>
+          <t>7.100142</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2283,7 +2259,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2298,12 +2274,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>9.99</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2313,7 +2289,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano 0</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2338,7 +2314,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2368,7 +2344,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126518</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>13.32</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,12 +2371,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2410,22 +2386,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>17.6089</t>
+          <t>8.36115</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3662</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1.5</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2450,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2480,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2490,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>48.078908</t>
+          <t>11.204221</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2507,27 +2483,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>33.06999</t>
+          <t>2.81507</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.7338</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2535,26 +2507,22 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2592,7 +2560,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2602,7 +2570,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>45.069833</t>
+          <t>11.204259</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2619,12 +2587,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2634,22 +2602,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>22.48</t>
+          <t>27.87055</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2674,7 +2642,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2704,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2714,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>48.085561</t>
+          <t>37.347471</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2731,39 +2699,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>9.38356</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano -0.5</t>
-        </is>
-      </c>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2786,7 +2746,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2816,7 +2776,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2826,7 +2786,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>48.067653</t>
+          <t>37.347502</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2843,12 +2803,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2858,22 +2818,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>11.42</t>
+          <t>12.87</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2898,7 +2858,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2928,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786117945</t>
+          <t>1786125953</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2938,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>24.427807</t>
+          <t>17.16</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2955,7 +2915,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2970,12 +2930,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>12.82</t>
+          <t>5.82</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2985,7 +2945,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2995,27 +2955,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3040,17 +3000,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786116567</t>
+          <t>1786124724</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>27.718919</t>
+          <t>15.836735</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3067,12 +3027,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3082,12 +3042,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6.27945</t>
+          <t>1.93998</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3152,7 +3112,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786124628</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3162,7 +3122,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>8.616741</t>
+          <t>2.58664</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3179,23 +3139,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.31576</t>
+          <t>3.55998</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3203,7 +3167,11 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3256,7 +3224,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786124356</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3266,7 +3234,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>8.616781</t>
+          <t>4.74664</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3283,12 +3251,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3298,22 +3266,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>27.21968</t>
+          <t>8.94</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3323,27 +3291,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3368,17 +3336,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786116497</t>
+          <t>1786123837</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>37.35119</t>
+          <t>24.080808</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3395,31 +3363,39 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.0374</t>
+          <t>17.66906</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Real Tomayapo -1</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3427,27 +3403,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3472,17 +3448,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786116493</t>
+          <t>1786123806</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>37.348465</t>
+          <t>48.079075</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3499,7 +3475,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3507,54 +3483,46 @@
           <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>27.12529</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>Real Oruro</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Real Tomayapo vs Real Oruro</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Real Tomayapo</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Real Oruro</t>
-        </is>
-      </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3584,7 +3552,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786116236</t>
+          <t>1786123085</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3594,7 +3562,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>62.947368</t>
+          <t>54.115292</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3611,31 +3579,39 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5075</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3643,27 +3619,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3688,17 +3664,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786116231</t>
+          <t>1786120674</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>79.82266</t>
+          <t>4.727273</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3715,7 +3691,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3730,12 +3706,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.85998</t>
+          <t>1.65998</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3800,7 +3776,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786115704</t>
+          <t>1786119912</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3810,7 +3786,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2.56549</t>
+          <t>2.25082</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3827,110 +3803,1654 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano 0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>17.6089</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.3662</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1.5</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>48.078908</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>33.06999</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.7338</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1786118876</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>45.069833</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22.48</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.4675</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1786118874</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>48.085561</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>28.42</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.5913</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -0.5</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1786118874</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>48.067653</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>11.42</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.4675</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1786117945</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>24.427807</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>12.82</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.4625</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1786116567</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>27.718919</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>6.27945</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>8.616741</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2.31576</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1786116498</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>8.616781</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>27.21968</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.7288</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1786116497</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>37.35119</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>10.0374</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.2688</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1786116493</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>37.348465</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>17.94</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1786116236</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>62.947368</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.5075</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1786116231</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>79.82266</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1.85998</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.725</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1786115704</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>2.56549</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>0x590b15150f41ddf420690c7cecb635a5facfe4448334123e390e09254607c190</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>9.19</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>1.3562</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Guabira</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>L19682540</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
         <is>
           <t>1786115704</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="S46" t="inlineStr">
         <is>
           <t>1786137300</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>25.796491</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-08 09:02:47 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Division Profesional/trades.xlsx
+++ b/data/sxbet/ligas/Division Profesional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x665ad5dc09f910a78682d8cac57b8941da70edf35f23f2fb6db3f128b63a18e8</t>
+          <t>0xe16eaff028990451968364aee83ca802c99521a40479400e0f271fcf1e623b4e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.31</t>
+          <t>1.00999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.8275</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>The Strongest</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>The Strongest vs Independiente Petrolero</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xb477e72b9ab6557e336768e8602ef1b40d5140beda07a5f9765228ca871d791f</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19692641</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786136236</t>
+          <t>1786178250</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786223700</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>19.374732</t>
+          <t>1.220532</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xf272c06e82de6d4f5a541673d36a6677e813d924b288c8fa65932e7f17a6e89f</t>
+          <t>0x778d5391d91c2202456bb2794070959085f92b254fb5e58d41ebde9406162bcb</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33.32</t>
+          <t>19.74</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +683,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>The Strongest vs Independiente Petrolero</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0x614c32809a7d6ad12c22c0256c9112ab22a296220275a1694649c55e7279b319</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19692641</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +728,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786136032</t>
+          <t>1786173034</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786223700</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>60.307692</t>
+          <t>272.275862</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,28 +755,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x0a6830dca2ddaafc8a77ba73c5db8e87d8f5fbc96d7d4d1fc85c80dd6a2dcff0</t>
+          <t>0x665ad5dc09f910a78682d8cac57b8941da70edf35f23f2fb6db3f128b63a18e8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>11.31</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -779,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786135821</t>
+          <t>1786136236</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>13.395349</t>
+          <t>19.374732</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,31 +859,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x1b16769a2446e95c5c45c0a5c1eee6a448ebe2fc2e9b698f501443da0dfe730a</t>
+          <t>0xf272c06e82de6d4f5a541673d36a6677e813d924b288c8fa65932e7f17a6e89f</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>33.32</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3538</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -898,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786135233</t>
+          <t>1786136032</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>8.961131</t>
+          <t>60.307692</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x3b7d6449f4a2a7f7e958feb31d1aa3512a36d932b93cd01aba4dae26404c5131</t>
+          <t>0x0a6830dca2ddaafc8a77ba73c5db8e87d8f5fbc96d7d4d1fc85c80dd6a2dcff0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -966,12 +982,12 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>17.00737</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3538</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -987,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1032,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786134933</t>
+          <t>1786135821</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>48.077371</t>
+          <t>13.395349</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x5b2bf2a561f9efc207b4be16204e262143fe9b1140ba536a8207f25e53ad496b</t>
+          <t>0x1b16769a2446e95c5c45c0a5c1eee6a448ebe2fc2e9b698f501443da0dfe730a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1070,12 +1086,12 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.22</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1091,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1136,17 +1152,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786134605</t>
+          <t>1786135233</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>5.431193</t>
+          <t>8.961131</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,39 +1179,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xcc60eac075cc4315d4dfa294b65cc4f174c2c9d458811a16d52e87b659d8ad45</t>
+          <t>0x3b7d6449f4a2a7f7e958feb31d1aa3512a36d932b93cd01aba4dae26404c5131</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>17.00737</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5362</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1218,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1248,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786134304</t>
+          <t>1786134933</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1258,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>9.323991</t>
+          <t>48.077371</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,39 +1283,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe21791ae1e8109a191bcf87ea7e050cf62a2cdf8ddab67d9bf182b3016b1b848</t>
+          <t>0x5b2bf2a561f9efc207b4be16204e262143fe9b1140ba536a8207f25e53ad496b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>2.22</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1315,27 +1315,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1360,17 +1360,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786134118</t>
+          <t>1786134605</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>49.767221</t>
+          <t>5.431193</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,12 +1387,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xc3316b5940ad1bd194feda7f00770a34f912831f1c7deace747e91137cafd11b</t>
+          <t>0xcc60eac075cc4315d4dfa294b65cc4f174c2c9d458811a16d52e87b659d8ad45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1402,22 +1402,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.16819</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3125</t>
+          <t>1.5362</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Over 4.5</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x48f1daf9c9d3e68c0ec6553b26f71366417addfa8f09d543cc8f8bdd0077b612</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786131200</t>
+          <t>1786134304</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>48.538208</t>
+          <t>9.323991</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,12 +1499,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x3c412198bcfc31cf640052941892a1f595f5547ec59a1414e24fbb1bfeb3ebae</t>
+          <t>0xe21791ae1e8109a191bcf87ea7e050cf62a2cdf8ddab67d9bf182b3016b1b848</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1514,22 +1514,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>18.5095</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.3813</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x2f4dc11491614174f697fd6856dc7dfbde0374f56c9c6b93da705d898b6b9392</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786131200</t>
+          <t>1786134118</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>48.549508</t>
+          <t>49.767221</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x2cb6bec7f2a474ec0b4c474043876d18add5eadb31632382e7e9f728fa247159</t>
+          <t>0xc3316b5940ad1bd194feda7f00770a34f912831f1c7deace747e91137cafd11b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1626,22 +1626,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15.66</t>
+          <t>15.16819</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6425</t>
+          <t>1.3125</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0x48f1daf9c9d3e68c0ec6553b26f71366417addfa8f09d543cc8f8bdd0077b612</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786131081</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>24.373541</t>
+          <t>48.538208</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x2a44ccf443a8d5632916aab67a3e7bc4147a268fe5d4978cedf712cfd7e2babf</t>
+          <t>0x3c412198bcfc31cf640052941892a1f595f5547ec59a1414e24fbb1bfeb3ebae</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1738,22 +1738,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>18.5095</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3838</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Nacional Potosí</t>
+          <t>Over 4.0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1763,27 +1763,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Nacional Potosí</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
+          <t>0x2f4dc11491614174f697fd6856dc7dfbde0374f56c9c6b93da705d898b6b9392</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19691489</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1808,17 +1808,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786130177</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2.605863</t>
+          <t>48.549508</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,12 +1835,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x116fd7242c980c72161b884392f42af79732e449e79f3dc7d212acd8ad8d658d</t>
+          <t>0x2cb6bec7f2a474ec0b4c474043876d18add5eadb31632382e7e9f728fa247159</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1850,22 +1850,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>15.66</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5088</t>
+          <t>1.6425</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786129447</t>
+          <t>1786131081</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>9.82799</t>
+          <t>24.373541</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,23 +1947,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xbbe9c61e5707bbf256b5c277314eeffa098594034d2dbb2bb99c6791f780e113</t>
+          <t>0x2a44ccf443a8d5632916aab67a3e7bc4147a268fe5d4978cedf712cfd7e2babf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.35999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1971,7 +1975,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Nacional Potosí</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2024,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786129377</t>
+          <t>1786130177</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>9.945932</t>
+          <t>2.605863</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,31 +2059,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
+          <t>0x116fd7242c980c72161b884392f42af79732e449e79f3dc7d212acd8ad8d658d</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2098,7 +2114,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2144,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786127516</t>
+          <t>1786129447</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2154,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>7.111111</t>
+          <t>9.82799</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2171,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
+          <t>0xbbe9c61e5707bbf256b5c277314eeffa098594034d2dbb2bb99c6791f780e113</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2166,17 +2182,17 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5.75999</t>
+          <t>7.35999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.8113</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2187,27 +2203,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>San Antonio Bulo Bulo</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19691489</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2232,17 +2248,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786127077</t>
+          <t>1786129377</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>7.100142</t>
+          <t>9.945932</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2259,7 +2275,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
+          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2267,46 +2283,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>9.99</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2314,7 +2322,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2344,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786126518</t>
+          <t>1786127516</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2354,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>13.32</t>
+          <t>7.111111</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2371,54 +2379,46 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
+          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>8.36115</t>
+          <t>5.75999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7462</t>
+          <t>1.8113</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786127077</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.204221</t>
+          <t>7.100142</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2483,23 +2483,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
+          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.81507</t>
+          <t>9.99</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.2512</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2507,7 +2511,11 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2560,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786126518</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2570,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>11.204259</t>
+          <t>13.32</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2587,7 +2595,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
+          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2602,7 +2610,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>27.87055</t>
+          <t>8.36115</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2672,7 +2680,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2682,7 +2690,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>37.347471</t>
+          <t>11.204221</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2699,7 +2707,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
+          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2710,7 +2718,7 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>9.38356</t>
+          <t>2.81507</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2776,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2786,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>37.347502</t>
+          <t>11.204259</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2803,12 +2811,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
+          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2818,12 +2826,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12.87</t>
+          <t>27.87055</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2888,7 +2896,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786125953</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2898,7 +2906,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>17.16</t>
+          <t>37.347471</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2915,39 +2923,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
+          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5.82</t>
+          <t>9.38356</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Real Tomayapo -1</t>
-        </is>
-      </c>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2955,27 +2955,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3000,17 +3000,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786124724</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>15.836735</t>
+          <t>37.347502</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3027,7 +3027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
+          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.93998</t>
+          <t>12.87</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786124628</t>
+          <t>1786125953</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2.58664</t>
+          <t>17.16</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3139,7 +3139,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
+          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3154,22 +3154,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.55998</t>
+          <t>5.82</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3179,27 +3179,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3224,17 +3224,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786124356</t>
+          <t>1786124724</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>4.74664</t>
+          <t>15.836735</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
+          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3266,22 +3266,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>8.94</t>
+          <t>1.93998</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3291,27 +3291,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3336,17 +3336,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786123837</t>
+          <t>1786124628</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>24.080808</t>
+          <t>2.58664</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3363,7 +3363,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
+          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3378,22 +3378,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>17.66906</t>
+          <t>3.55998</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3403,27 +3403,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3448,17 +3448,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786123806</t>
+          <t>1786124356</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>48.079075</t>
+          <t>4.74664</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,31 +3475,39 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
+          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>27.12529</t>
+          <t>8.94</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Real Tomayapo -1</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3522,7 +3530,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3552,7 +3560,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786123085</t>
+          <t>1786123837</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3562,7 +3570,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>54.115292</t>
+          <t>24.080808</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3579,7 +3587,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
+          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3594,22 +3602,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>17.66906</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.7425</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3619,27 +3627,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3664,17 +3672,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786120674</t>
+          <t>1786123806</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>4.727273</t>
+          <t>48.079075</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3691,39 +3699,31 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
+          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.65998</t>
+          <t>27.12529</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.7375</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3731,27 +3731,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3776,17 +3776,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786119912</t>
+          <t>1786123085</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2.25082</t>
+          <t>54.115292</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,7 +3803,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano 0</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786120674</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4.727273</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,7 +3915,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3930,22 +3930,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>17.6089</t>
+          <t>1.65998</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.3662</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1.5</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786119912</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>48.078908</t>
+          <t>2.25082</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,7 +4027,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4042,12 +4042,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>33.06999</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7338</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4057,24 +4057,24 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano 0</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>45.069833</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4154,22 +4154,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>22.48</t>
+          <t>17.6089</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.3662</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>48.085561</t>
+          <t>48.078908</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,7 +4251,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4266,22 +4266,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>33.06999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.7338</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -0.5</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>48.067653</t>
+          <t>45.069833</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,12 +4363,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>11.42</t>
+          <t>22.48</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786117945</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>24.427807</t>
+          <t>48.085561</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4490,22 +4490,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>12.82</t>
+          <t>28.42</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano -0.5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786116567</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>27.718919</t>
+          <t>48.067653</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4587,12 +4587,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4602,39 +4602,39 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>6.27945</t>
+          <t>11.42</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.4675</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786117945</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>8.616741</t>
+          <t>24.427807</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4699,31 +4699,39 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2.31576</t>
+          <t>12.82</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.4625</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -4746,7 +4754,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4776,7 +4784,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786116567</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4786,7 +4794,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>8.616781</t>
+          <t>27.718919</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4803,7 +4811,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4818,7 +4826,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>27.21968</t>
+          <t>6.27945</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4888,7 +4896,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786116497</t>
+          <t>1786116498</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4898,7 +4906,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>37.35119</t>
+          <t>8.616741</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4915,7 +4923,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4926,7 +4934,7 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.0374</t>
+          <t>2.31576</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4992,7 +5000,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786116493</t>
+          <t>1786116498</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5002,7 +5010,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>37.348465</t>
+          <t>8.616781</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5019,12 +5027,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5034,22 +5042,22 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>27.21968</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.7288</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -5059,27 +5067,27 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -5104,17 +5112,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786116236</t>
+          <t>1786116497</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>62.947368</t>
+          <t>37.35119</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5131,28 +5139,28 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>10.0374</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.5075</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -5163,27 +5171,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5208,17 +5216,17 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786116231</t>
+          <t>1786116493</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>79.82266</t>
+          <t>37.348465</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5235,12 +5243,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5250,22 +5258,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.85998</t>
+          <t>17.94</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.285</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -5275,27 +5283,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5320,17 +5328,17 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786115704</t>
+          <t>1786116236</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2.56549</t>
+          <t>62.947368</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5347,110 +5355,326 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.5075</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1786116231</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>79.82266</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>1.85998</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.725</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1786115704</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>2.56549</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>0x590b15150f41ddf420690c7cecb635a5facfe4448334123e390e09254607c190</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>9.19</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>1.3562</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Guabira</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>L19682540</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr">
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
         <is>
           <t>1786115704</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t>1786137300</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>25.796491</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-08 12:02:29 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Division Profesional/trades.xlsx
+++ b/data/sxbet/ligas/Division Profesional/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,27 +531,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe16eaff028990451968364aee83ca802c99521a40479400e0f271fcf1e623b4e</t>
+          <t>0xf39343d92792a4f591dfeab72647abe656b994a66927bfb38db6f88c28d9259b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.00999</t>
+          <t>11.66</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.8275</t>
+          <t>1.2312</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -559,26 +555,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>The Strongest vs Independiente Petrolero</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>The Strongest</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>The Strongest vs Independiente Petrolero</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>The Strongest</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Independiente Petrolero</t>
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786178250</t>
+          <t>1786189746</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.220532</t>
+          <t>50.421622</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,27 +635,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x778d5391d91c2202456bb2794070959085f92b254fb5e58d41ebde9406162bcb</t>
+          <t>0xaa73d02b6f6462028f4aaf2a1f2453c2457b7b1fcb67bda7fc70f3a8fa759652</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19.74</t>
+          <t>1.76989</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.935</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -671,31 +659,27 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>The Strongest vs Independiente Petrolero</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>The Strongest</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Independiente Petrolero</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>The Strongest vs Independiente Petrolero</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>The Strongest</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Independiente Petrolero</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>0x614c32809a7d6ad12c22c0256c9112ab22a296220275a1694649c55e7279b319</t>
@@ -728,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786173034</t>
+          <t>1786187481</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>272.275862</t>
+          <t>1.89293</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,28 +739,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x665ad5dc09f910a78682d8cac57b8941da70edf35f23f2fb6db3f128b63a18e8</t>
+          <t>0xa3e049b9059bc91013a03aaa8ab9db007b42c2067a464c3861cb1b7ceb2f4518</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11.31</t>
+          <t>21.125</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.2112</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -787,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>The Strongest vs Independiente Petrolero</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xb477e72b9ab6557e336768e8602ef1b40d5140beda07a5f9765228ca871d791f</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19692641</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786136236</t>
+          <t>1786182543</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786223700</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>19.374732</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +843,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xf272c06e82de6d4f5a541673d36a6677e813d924b288c8fa65932e7f17a6e89f</t>
+          <t>0xe16eaff028990451968364aee83ca802c99521a40479400e0f271fcf1e623b4e</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,22 +858,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>33.32</t>
+          <t>1.00999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.8275</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>The Strongest vs Independiente Petrolero</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xb477e72b9ab6557e336768e8602ef1b40d5140beda07a5f9765228ca871d791f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19692641</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786136032</t>
+          <t>1786178250</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786223700</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>60.307692</t>
+          <t>1.220532</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,31 +955,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x0a6830dca2ddaafc8a77ba73c5db8e87d8f5fbc96d7d4d1fc85c80dd6a2dcff0</t>
+          <t>0x778d5391d91c2202456bb2794070959085f92b254fb5e58d41ebde9406162bcb</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>19.74</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Independiente Petrolero</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1003,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>The Strongest vs Independiente Petrolero</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>The Strongest</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Independiente Petrolero</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
+          <t>0x614c32809a7d6ad12c22c0256c9112ab22a296220275a1694649c55e7279b319</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19692641</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1040,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786135821</t>
+          <t>1786173034</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786223700</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>13.395349</t>
+          <t>272.275862</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,28 +1067,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x1b16769a2446e95c5c45c0a5c1eee6a448ebe2fc2e9b698f501443da0dfe730a</t>
+          <t>0x665ad5dc09f910a78682d8cac57b8941da70edf35f23f2fb6db3f128b63a18e8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>11.31</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3538</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1122,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786135233</t>
+          <t>1786136236</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>8.961131</t>
+          <t>19.374732</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,31 +1171,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x3b7d6449f4a2a7f7e958feb31d1aa3512a36d932b93cd01aba4dae26404c5131</t>
+          <t>0xf272c06e82de6d4f5a541673d36a6677e813d924b288c8fa65932e7f17a6e89f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17.00737</t>
+          <t>33.32</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3538</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786134933</t>
+          <t>1786136032</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>48.077371</t>
+          <t>60.307692</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x5b2bf2a561f9efc207b4be16204e262143fe9b1140ba536a8207f25e53ad496b</t>
+          <t>0x0a6830dca2ddaafc8a77ba73c5db8e87d8f5fbc96d7d4d1fc85c80dd6a2dcff0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1294,12 +1294,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.22</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786134605</t>
+          <t>1786135821</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>5.431193</t>
+          <t>13.395349</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,39 +1387,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xcc60eac075cc4315d4dfa294b65cc4f174c2c9d458811a16d52e87b659d8ad45</t>
+          <t>0x1b16769a2446e95c5c45c0a5c1eee6a448ebe2fc2e9b698f501443da0dfe730a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5362</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1442,7 +1434,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1472,7 +1464,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786134304</t>
+          <t>1786135233</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1474,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>9.323991</t>
+          <t>8.961131</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,39 +1491,31 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xe21791ae1e8109a191bcf87ea7e050cf62a2cdf8ddab67d9bf182b3016b1b848</t>
+          <t>0x3b7d6449f4a2a7f7e958feb31d1aa3512a36d932b93cd01aba4dae26404c5131</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>17.00737</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5263</t>
+          <t>1.3538</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1554,7 +1538,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1568,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786134118</t>
+          <t>1786134933</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1578,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>49.767221</t>
+          <t>48.077371</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xc3316b5940ad1bd194feda7f00770a34f912831f1c7deace747e91137cafd11b</t>
+          <t>0x5b2bf2a561f9efc207b4be16204e262143fe9b1140ba536a8207f25e53ad496b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1619,31 +1603,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15.16819</t>
+          <t>2.22</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3125</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -1651,27 +1627,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x48f1daf9c9d3e68c0ec6553b26f71366417addfa8f09d543cc8f8bdd0077b612</t>
+          <t>0xd3779282ef9e4691761048b5151f1cb89c2b98e8b99d1ab7e6e6c64113635260</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1696,17 +1672,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786131200</t>
+          <t>1786134605</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>48.538208</t>
+          <t>5.431193</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,12 +1699,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x3c412198bcfc31cf640052941892a1f595f5547ec59a1414e24fbb1bfeb3ebae</t>
+          <t>0xcc60eac075cc4315d4dfa294b65cc4f174c2c9d458811a16d52e87b659d8ad45</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1738,22 +1714,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>18.5095</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3813</t>
+          <t>1.5362</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1778,7 +1754,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x2f4dc11491614174f697fd6856dc7dfbde0374f56c9c6b93da705d898b6b9392</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1808,7 +1784,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786131200</t>
+          <t>1786134304</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1794,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>48.549508</t>
+          <t>9.323991</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,12 +1811,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x2cb6bec7f2a474ec0b4c474043876d18add5eadb31632382e7e9f728fa247159</t>
+          <t>0xe21791ae1e8109a191bcf87ea7e050cf62a2cdf8ddab67d9bf182b3016b1b848</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1850,22 +1826,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.66</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.6425</t>
+          <t>1.5263</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1890,7 +1866,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1920,7 +1896,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786131081</t>
+          <t>1786134118</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1906,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>24.373541</t>
+          <t>49.767221</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,12 +1923,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x2a44ccf443a8d5632916aab67a3e7bc4147a268fe5d4978cedf712cfd7e2babf</t>
+          <t>0xc3316b5940ad1bd194feda7f00770a34f912831f1c7deace747e91137cafd11b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1962,22 +1938,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.16819</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3838</t>
+          <t>1.3125</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Nacional Potosí</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1987,27 +1963,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Nacional Potosí</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
+          <t>0x48f1daf9c9d3e68c0ec6553b26f71366417addfa8f09d543cc8f8bdd0077b612</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19691489</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2032,17 +2008,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786130177</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2.605863</t>
+          <t>48.538208</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2059,12 +2035,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x116fd7242c980c72161b884392f42af79732e449e79f3dc7d212acd8ad8d658d</t>
+          <t>0x3c412198bcfc31cf640052941892a1f595f5547ec59a1414e24fbb1bfeb3ebae</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2074,22 +2050,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4.99999</t>
+          <t>18.5095</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5088</t>
+          <t>1.3813</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 4.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2114,7 +2090,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
+          <t>0x2f4dc11491614174f697fd6856dc7dfbde0374f56c9c6b93da705d898b6b9392</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2144,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786129447</t>
+          <t>1786131200</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2154,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>9.82799</t>
+          <t>48.549508</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2171,7 +2147,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xbbe9c61e5707bbf256b5c277314eeffa098594034d2dbb2bb99c6791f780e113</t>
+          <t>0x2cb6bec7f2a474ec0b4c474043876d18add5eadb31632382e7e9f728fa247159</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2179,23 +2155,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>7.35999</t>
+          <t>15.66</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.6425</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2203,27 +2187,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>San Antonio Bulo Bulo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Nacional Potosí</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
+          <t>0x491ded7835f0cda7922dee91d1cbc277b69bb5da61c7be630a919284af357592</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19691489</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2248,17 +2232,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786129377</t>
+          <t>1786131081</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786215600</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>9.945932</t>
+          <t>24.373541</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,31 +2259,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
+          <t>0x2a44ccf443a8d5632916aab67a3e7bc4147a268fe5d4978cedf712cfd7e2babf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.3838</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Nacional Potosí</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2307,27 +2299,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>San Antonio Bulo Bulo</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19691489</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2352,17 +2344,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786127516</t>
+          <t>1786130177</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>7.111111</t>
+          <t>2.605863</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2379,31 +2371,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
+          <t>0x116fd7242c980c72161b884392f42af79732e449e79f3dc7d212acd8ad8d658d</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.75999</t>
+          <t>4.99999</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.8113</t>
+          <t>1.5088</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
+          <t>0x0e1c46a583926b3308cdb91be9a4c98f1faa27ed00668e5a3022fd06f96adbfb</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786127077</t>
+          <t>1786129447</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>7.100142</t>
+          <t>9.82799</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2483,7 +2483,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
+          <t>0xbbe9c61e5707bbf256b5c277314eeffa098594034d2dbb2bb99c6791f780e113</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2491,31 +2491,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9.99</t>
+          <t>7.35999</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -2523,27 +2515,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>San Antonio Bulo Bulo vs Nacional Potosí</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>San Antonio Bulo Bulo</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Nacional Potosí</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x911bd51e46175fe9d225b374da8c9683813fac3a6ae307652700b382561964f3</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19691489</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2568,17 +2560,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786126518</t>
+          <t>1786129377</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786215600</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>13.32</t>
+          <t>9.945932</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2595,54 +2587,46 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
+          <t>0xa62f250ff2f43c3bb34525d562a9f70e050c859e38dc19adf04adae248a4e98f</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>8.36115</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.7462</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -2650,7 +2634,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2680,7 +2664,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786127516</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2690,7 +2674,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>11.204221</t>
+          <t>7.111111</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2707,28 +2691,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
+          <t>0x0858011830e20e0cbfb1e43413cbd279d8984110bee80f2ae61ebfad9aaa0ab8</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.81507</t>
+          <t>5.75999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2512</t>
+          <t>1.8113</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2754,7 +2738,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x68ad1bb7e88acbf83c09926e656f505fd89df351ed43ff1e7aad919a2d0cdaae</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2784,7 +2768,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786126508</t>
+          <t>1786127077</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2794,7 +2778,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>11.204259</t>
+          <t>7.100142</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2811,12 +2795,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
+          <t>0x5011867ed5b463eaca1c24497bfc1f7d948a9bc0c26c70c9d852755682ba6eee</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2826,12 +2810,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>27.87055</t>
+          <t>9.99</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.7462</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2896,7 +2880,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786126518</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2906,7 +2890,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>37.347471</t>
+          <t>13.32</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2923,7 +2907,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
+          <t>0xb6e0812ef93e960870c52f2f1faf333136580d28861d47fde2e61935f3860f12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2931,15 +2915,19 @@
           <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>9.38356</t>
+          <t>8.36115</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2512</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2947,7 +2935,11 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3000,7 +2992,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786126505</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3010,7 +3002,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>37.347502</t>
+          <t>11.204221</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3027,27 +3019,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
+          <t>0x9bd982e33d22074983f5138991b39dc45e478934065574d7b45b291bc084485e</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>12.87</t>
+          <t>2.81507</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3055,26 +3043,22 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -3112,7 +3096,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786125953</t>
+          <t>1786126508</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3122,7 +3106,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>17.16</t>
+          <t>11.204259</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3139,12 +3123,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
+          <t>0xc38ae621d8fca720bddf8fcfb0463c1e1a390ff07c8c974251d96d1ae7fb7c56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3154,22 +3138,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.82</t>
+          <t>27.87055</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.7462</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3179,27 +3163,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3224,17 +3208,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786124724</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>15.836735</t>
+          <t>37.347471</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3251,27 +3235,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
+          <t>0x0368c1bb4d6609c35c97b48075e98b9d2c4222ddf6302ab88136e3741e6ce3a5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.93998</t>
+          <t>9.38356</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.2512</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3279,26 +3259,22 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -3336,7 +3312,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786124628</t>
+          <t>1786126505</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3346,7 +3322,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2.58664</t>
+          <t>37.347502</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3363,7 +3339,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
+          <t>0x7f8f46466701fdfddd757f918f5a804848fbc67ad4bdcec366e181e3d16f1b3d</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3378,7 +3354,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3.55998</t>
+          <t>12.87</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3448,7 +3424,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786124356</t>
+          <t>1786125953</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3458,7 +3434,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>4.74664</t>
+          <t>17.16</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,7 +3451,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
+          <t>0xa73a2931f37ee8369aa2d183c637aac54b2917f644d1011c5108ce866cbac8f8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3490,12 +3466,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>8.94</t>
+          <t>5.82</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3713</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3560,7 +3536,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786123837</t>
+          <t>1786124724</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3570,7 +3546,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>24.080808</t>
+          <t>15.836735</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,7 +3563,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
+          <t>0x7615a3a9a5753889a9bd269dd030cc5e94939d5600ca1a6b6d0287f8bf9fc8f5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3602,22 +3578,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>17.66906</t>
+          <t>1.93998</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Real Tomayapo -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3627,27 +3603,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3672,17 +3648,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786123806</t>
+          <t>1786124628</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>48.079075</t>
+          <t>2.58664</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,31 +3675,39 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
+          <t>0x4e4b1dcf666f51909f26dc3ba295c4d3aaa5538529e00c4032af14f9cffe430d</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>27.12529</t>
+          <t>3.55998</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5012</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -3731,27 +3715,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3776,17 +3760,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786123085</t>
+          <t>1786124356</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>54.115292</t>
+          <t>4.74664</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,7 +3787,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
+          <t>0x862b8ed2cf92c8393495af2afc0f5837c31b91839af481202ed412f03bf8971b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3818,22 +3802,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>8.94</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.7425</t>
+          <t>1.3713</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3843,27 +3827,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3888,17 +3872,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786120674</t>
+          <t>1786123837</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>4.727273</t>
+          <t>24.080808</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,7 +3899,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
+          <t>0x3664cb675bf0848a30ca29bb1a35549acf19d0f40c4fc6c013d8aa481af892b0</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3930,22 +3914,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.65998</t>
+          <t>17.66906</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.7375</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo -1</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3955,27 +3939,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb9da4c9ca0557d27b99a185a3800d8d469d1bad868c55fdb946cd65a6065a888</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4000,17 +3984,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786119912</t>
+          <t>1786123806</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2.25082</t>
+          <t>48.079075</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,39 +4011,31 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
+          <t>0x467eb043a2e00a48349804e6ea64170cacb13197d8f53b68cdba9b4fecbda5c2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>27.12529</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.5012</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano 0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -4067,27 +4043,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
+          <t>Real Tomayapo vs Real Oruro</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano</t>
+          <t>Real Tomayapo</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Guabira</t>
+          <t>Real Oruro</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
+          <t>0xf8758bfa74fe88e8b3ae46990bfd7fdc85028fe092095742999df545e0a58e73</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19682540</t>
+          <t>L19683272</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4112,17 +4088,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786123085</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1786137300</t>
+          <t>1786145400</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>54.115292</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4139,7 +4115,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
+          <t>0xfb8706347229edbfbecceb1ec967cad8f2155ba3564efd2f9b129bdf52053cdd</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4154,22 +4130,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>17.6089</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.3662</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1.5</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4194,7 +4170,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4224,7 +4200,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786120674</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4234,7 +4210,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>48.078908</t>
+          <t>4.727273</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4251,7 +4227,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
+          <t>0x5c61b658ed160e256a1a04509c60d05282cca9ee175f758004726d00cda9fda3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4266,12 +4242,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>33.06999</t>
+          <t>1.65998</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.7338</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4336,7 +4312,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786118876</t>
+          <t>1786119912</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4346,7 +4322,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>45.069833</t>
+          <t>2.25082</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4363,7 +4339,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
+          <t>0xf5bbffb37c6e30c4b29c9b786f1d3cbc6312852512b5f5b8d7e546953f1d5d41</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4378,22 +4354,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>22.48</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano 0</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4418,7 +4394,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xf2dc7e574dbabb1bf692c4f4ee6e476cf533cc7b889ce2c4d27bf689231ae30b</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4448,7 +4424,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4458,7 +4434,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>48.085561</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4475,7 +4451,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
+          <t>0x937fccf05d1a03c61c6c49ecc4f09bfa4458fe95c68d2576b5936782adbdf745</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4490,22 +4466,22 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>17.6089</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.3662</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -0.5</t>
+          <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4530,7 +4506,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
+          <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4560,7 +4536,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786118874</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4570,7 +4546,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>48.067653</t>
+          <t>48.078908</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4587,12 +4563,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
+          <t>0x2bdb8d570c912295736becb6fb2d2e8ac3dd6846d901ec5dec62742a8fe36302</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4602,22 +4578,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>11.42</t>
+          <t>33.06999</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.4675</t>
+          <t>1.7338</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Division Profesional</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Academia De Balompie Boliviano -1</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4642,7 +4618,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4672,7 +4648,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1786117945</t>
+          <t>1786118876</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4682,7 +4658,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>24.427807</t>
+          <t>45.069833</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4699,7 +4675,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
+          <t>0x7fae1c283411af3a5d69339f0766d48c13455376b26c65fa4f1b543f0542dc68</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4714,12 +4690,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>12.82</t>
+          <t>22.48</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.4625</t>
+          <t>1.4675</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4784,7 +4760,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1786116567</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4794,7 +4770,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>27.718919</t>
+          <t>48.085561</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4811,12 +4787,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
+          <t>0x2f90ba886d93902d9eceebc807f893a7a79859ea55117da82a029f6e15a67ffb</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4826,39 +4802,39 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>6.27945</t>
+          <t>28.42</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano -0.5</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -4866,7 +4842,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0xb76db3bf5b6df2ca9673c137392f1227cb428d254d2b85ceaf7ff3c093456f4d</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4896,7 +4872,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786118874</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4906,7 +4882,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>8.616741</t>
+          <t>48.067653</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4923,31 +4899,39 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
+          <t>0x74a826ebfcfd5acb3a91baef87b2df562f10cbb9bdd3b492bbdb0b00c46c9690</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2.31576</t>
+          <t>11.42</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.4675</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -4970,7 +4954,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -5000,7 +4984,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1786116498</t>
+          <t>1786117945</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -5010,7 +4994,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>8.616781</t>
+          <t>24.427807</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -5027,12 +5011,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
+          <t>0xc807431dabca948a7eef7c0732e33166de0f9e9ccf237561c91240f8840da1ec</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5042,39 +5026,39 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>27.21968</t>
+          <t>12.82</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.7288</t>
+          <t>1.4625</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Division Profesional</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
+          <t>Academia De Balompie Boliviano -1</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K43" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -5082,7 +5066,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+          <t>0x224d1b4bc2b57cc5978d2922e84bc81203465c5fd8cbeb4422d303fd7c400f1e</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5112,7 +5096,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1786116497</t>
+          <t>1786116567</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5122,7 +5106,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>37.35119</t>
+          <t>27.718919</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5139,7 +5123,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
+          <t>0xa0e42ac580f9d658c876264fdfce46a01d75892392accefaecd1d3bc438d404e</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5147,15 +5131,19 @@
           <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.0374</t>
+          <t>6.27945</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.2688</t>
+          <t>1.7288</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5163,7 +5151,11 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -5216,7 +5208,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1786116493</t>
+          <t>1786116498</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5226,7 +5218,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>37.348465</t>
+          <t>8.616741</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5243,39 +5235,31 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+          <t>0x09e6762fac3afbc9893a9380f32b25cbcc92464d9c11ccbcf1f5d67068ea89c7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>2.31576</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Real Oruro</t>
-        </is>
-      </c>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -5283,27 +5267,27 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5328,17 +5312,17 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1786116236</t>
+          <t>1786116498</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>62.947368</t>
+          <t>8.616781</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5355,31 +5339,39 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+          <t>0xd1a47102f15e31997aed9d1f25b0658b9e0366499701d5990eebc4b8bb72dd8e</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>27.21968</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.5075</t>
+          <t>1.7288</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>Division Profesional</t>
@@ -5387,27 +5379,27 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Real Tomayapo vs Real Oruro</t>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Real Tomayapo</t>
+          <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Real Oruro</t>
+          <t>Guabira</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>L19683272</t>
+          <t>L19682540</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -5432,17 +5424,17 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1786116231</t>
+          <t>1786116497</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>1786145400</t>
+          <t>1786137300</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>79.82266</t>
+          <t>37.35119</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5459,27 +5451,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+          <t>0x75feb6c5e98d8cc369d1dbddf86b8415299f2b3736a92898e07569169c537528</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xF544c218C0Ba0BAfD9Dd049E469097AE58B235c2</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>1.85998</t>
+          <t>10.0374</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.2688</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5487,26 +5475,22 @@
           <t>Division Profesional</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano vs Guabira</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>Academia De Balompie Boliviano</t>
-        </is>
-      </c>
       <c r="K47" t="inlineStr">
         <is>
           <t>Guabira</t>
@@ -5544,7 +5528,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1786115704</t>
+          <t>1786116493</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -5554,7 +5538,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>2.56549</t>
+          <t>37.348465</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5571,110 +5555,438 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0x232a1a673706827257f912fbf14de856ef17bdfcbab1a07ac3ada89a596e5d9f</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>17.94</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.285</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0xb3ce5682da68ef1a586a9b07396d45e2457b987b733027163106acc3835c384c</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1786116236</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>62.947368</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0x34c5fcd3f87a29f4e7bcccb0185ce177b86875bd2aca2067492a8c5c5e51f6e8</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x9B0B1AFA7bDED657DA5de911b1772ABe95e83290</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.5075</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Real Oruro</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Real Tomayapo</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x03ab73c7b230138be63e39afa73d391ca5ebdd8a3f3d3b5e399ee1cd32fa1040</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19683272</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1786116231</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1786145400</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>79.82266</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0x80cde5b15660e5fc13a5df47d634f99902cb234d188fab5ab215a1da84844d7e</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1.85998</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.725</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano vs Guabira</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Academia De Balompie Boliviano</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Guabira</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0xcd2fd1966093a1babd5bc256363d39e156a4dde6e33bbe69c5f2fd48c0a27f3c</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19682540</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1786115704</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1786137300</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>2.56549</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>0x590b15150f41ddf420690c7cecb635a5facfe4448334123e390e09254607c190</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>9.19</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>1.3562</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano -1.5</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Division Profesional</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Division Profesional</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano vs Guabira</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>Academia De Balompie Boliviano</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>Guabira</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>0x861fbd464f94d528425eae758a57be7858924dd394418e99816cd4e1df5841dd</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="M51" t="inlineStr">
         <is>
           <t>L19682540</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
         <is>
           <t>1786115704</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S51" t="inlineStr">
         <is>
           <t>1786137300</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T51" t="inlineStr">
         <is>
           <t>25.796491</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
+      <c r="V51" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>